<commit_message>
results based on simulated data updated
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Tabella_2_asl_2025/g_output/D6_Table_2_CE.xlsx
+++ b/i_test/test_D6_Tabella_2_asl_2025/g_output/D6_Table_2_CE.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -374,7 +374,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1649</t>
+          <t>1629</t>
         </is>
       </c>
     </row>
@@ -388,72 +388,120 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>A10BD</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1.638 (99,3%)</t>
+          <t>A10BD B10BD C10BD C10BX C10CE 6 (0,4%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A10AE</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>858 (52,0%)</t>
+          <t>A10BD B10BD C10BD C10BH C10CE 5 (0,3%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A10BH</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>526 (31,9%)</t>
+          <t>A10BD A10BX B10BD C10BD C10CE 5 (0,3%)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A10BK</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>500 (30,3%)</t>
+          <t>A10AE A10BD B10BD B10BJ C10BD C10CE 5 (0,3%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A10BJ</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>467 (28,3%)</t>
+          <t>A10BD B10AE B10BD B10BJ C10BD 5 (0,3%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A10BX</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>453 (27,5%)</t>
+          <t>A10BD B10BD B10BE C10BD C10CE 5 (0,3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>A10BD A10BK B10BD C10BD C10BK 5 (0,3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>A10BD B10BD B10BJ C10BD C10CE 5 (0,3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>A10AE A10BD B10BD B10BE C10BD 4 (0,2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>A10BD B10BD C10BD C10BJ C10BX 4 (0,2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated results based on simulated data uploaded
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Tabella_2_asl_2025/g_output/D6_Table_2_CE.xlsx
+++ b/i_test/test_D6_Tabella_2_asl_2025/g_output/D6_Table_2_CE.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -381,7 +381,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Combinazioni ATC IV livello (*)</t>
+          <t>Combinazioni di ≥5 ATC IV livello (*)</t>
         </is>
       </c>
     </row>
@@ -393,7 +393,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A10BD B10BD C10BD C10BX C10CE 6 (0,4%)</t>
+          <t>d a B10BD C10BD N15CE 24 (1,5%)</t>
         </is>
       </c>
     </row>
@@ -405,7 +405,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A10BD B10BD C10BD C10BH C10CE 5 (0,3%)</t>
+          <t>a B10BD C10BD C10CE N11BD 24 (1,5%)</t>
         </is>
       </c>
     </row>
@@ -417,7 +417,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A10BD A10BX B10BD C10BD C10CE 5 (0,3%)</t>
+          <t>d a B10BD C10BD C10CE 23 (1,4%)</t>
         </is>
       </c>
     </row>
@@ -429,7 +429,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>A10AE A10BD B10BD B10BJ C10BD C10CE 5 (0,3%)</t>
+          <t>d a B10BD C10BD D15CE 23 (1,4%)</t>
         </is>
       </c>
     </row>
@@ -441,7 +441,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>A10BD B10AE B10BD B10BJ C10BD 5 (0,3%)</t>
+          <t>d a B10BD C10BD J01BK 23 (1,4%)</t>
         </is>
       </c>
     </row>
@@ -453,7 +453,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A10BD B10BD B10BE C10BD C10CE 5 (0,3%)</t>
+          <t>a B10BD C10BD C10CE N05BD 23 (1,4%)</t>
         </is>
       </c>
     </row>
@@ -465,7 +465,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A10BD A10BK B10BD C10BD C10BK 5 (0,3%)</t>
+          <t>a B10BD C10BD C10CE N17BD 23 (1,4%)</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A10BD B10BD B10BJ C10BD C10CE 5 (0,3%)</t>
+          <t>d a B10BD C10BD D19BD 22 (1,4%)</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>A10AE A10BD B10BD B10BE C10BD 4 (0,2%)</t>
+          <t>a B10BD C10BD C10CE J15CE 22 (1,4%)</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,134 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>A10BD B10BD C10BD C10BJ C10BX 4 (0,2%)</t>
+          <t>a B10BD C10BD C10CE N15CE 22 (1,4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Combinazioni di ≥10 ATC IV livello (*)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>a d a B10BD C10BD C10BJ C10CE D08BD N01BK N11BD 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD C10BJ D03BX J02BJ J13BD J19BD N13BD N15CE 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD C10BJ D10D1 D12BD D15CE J02BJ J07BD J19BD 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD C10BJ D10D1 D12BD D15CE J02BJ J07BD N04BH 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD C10BJ D10D1 D12BD D15CE J02BJ J19BD N04BH 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD C10BJ D10D1 D12BD D15CE J07BD J19BD N04BH 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD C10BJ D10D1 D12BD J02BJ J07BD J19BD N04BH 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD C10BJ D10D1 D15CE J02BJ J07BD J19BD N04BH 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD C10BJ D12BD D15CE J02BJ J07BD J19BD N04BH 2 (0,1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>a B10BD C10BD D04BH D10D1 J05BD J08BD J13BD J14CE N12BD 2 (0,1%)</t>
         </is>
       </c>
     </row>

</xml_diff>